<commit_message>
No of Count Days Updated
</commit_message>
<xml_diff>
--- a/dataentry/uploaded_excel_files/cgle_2019_kyas.xlsx
+++ b/dataentry/uploaded_excel_files/cgle_2019_kyas.xlsx
@@ -3475,9 +3475,6 @@
     <t>10000000106</t>
   </si>
   <si>
-    <t>10000000122</t>
-  </si>
-  <si>
     <t>10000000134</t>
   </si>
   <si>
@@ -3785,6 +3782,9 @@
   </si>
   <si>
     <t>10000002073</t>
+  </si>
+  <si>
+    <t>10000863847</t>
   </si>
 </sst>
 </file>
@@ -3817,9 +3817,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4124,6 +4125,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S108"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
@@ -4344,8 +4348,8 @@
       </c>
     </row>
     <row r="5" spans="1:19">
-      <c r="A5" s="1" t="s">
-        <v>1153</v>
+      <c r="A5" s="2" t="s">
+        <v>1256</v>
       </c>
       <c r="B5" t="s">
         <v>26</v>
@@ -4398,7 +4402,7 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" s="1" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="B6" t="s">
         <v>26</v>
@@ -4451,7 +4455,7 @@
     </row>
     <row r="7" spans="1:19">
       <c r="A7" s="1" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="B7" t="s">
         <v>26</v>
@@ -4504,7 +4508,7 @@
     </row>
     <row r="8" spans="1:19">
       <c r="A8" s="1" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="B8" t="s">
         <v>26</v>
@@ -4557,7 +4561,7 @@
     </row>
     <row r="9" spans="1:19">
       <c r="A9" s="1" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="B9" t="s">
         <v>26</v>
@@ -4610,7 +4614,7 @@
     </row>
     <row r="10" spans="1:19">
       <c r="A10" s="1" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="B10" t="s">
         <v>26</v>
@@ -4663,7 +4667,7 @@
     </row>
     <row r="11" spans="1:19">
       <c r="A11" s="1" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="B11" t="s">
         <v>26</v>
@@ -4716,7 +4720,7 @@
     </row>
     <row r="12" spans="1:19">
       <c r="A12" s="1" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="B12" t="s">
         <v>26</v>
@@ -4769,7 +4773,7 @@
     </row>
     <row r="13" spans="1:19">
       <c r="A13" s="1" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="B13" t="s">
         <v>26</v>
@@ -4822,7 +4826,7 @@
     </row>
     <row r="14" spans="1:19">
       <c r="A14" s="1" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="B14" t="s">
         <v>26</v>
@@ -4875,7 +4879,7 @@
     </row>
     <row r="15" spans="1:19">
       <c r="A15" s="1" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="B15" t="s">
         <v>26</v>
@@ -4928,7 +4932,7 @@
     </row>
     <row r="16" spans="1:19">
       <c r="A16" s="1" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="B16" t="s">
         <v>26</v>
@@ -4981,7 +4985,7 @@
     </row>
     <row r="17" spans="1:19">
       <c r="A17" s="1" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="B17" t="s">
         <v>26</v>
@@ -5034,7 +5038,7 @@
     </row>
     <row r="18" spans="1:19">
       <c r="A18" s="1" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="B18" t="s">
         <v>26</v>
@@ -5087,7 +5091,7 @@
     </row>
     <row r="19" spans="1:19">
       <c r="A19" s="1" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="B19" t="s">
         <v>26</v>
@@ -5140,7 +5144,7 @@
     </row>
     <row r="20" spans="1:19">
       <c r="A20" s="1" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="B20" t="s">
         <v>26</v>
@@ -5193,7 +5197,7 @@
     </row>
     <row r="21" spans="1:19">
       <c r="A21" s="1" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="B21" t="s">
         <v>26</v>
@@ -5246,7 +5250,7 @@
     </row>
     <row r="22" spans="1:19">
       <c r="A22" s="1" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="B22" t="s">
         <v>26</v>
@@ -5299,7 +5303,7 @@
     </row>
     <row r="23" spans="1:19">
       <c r="A23" s="1" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="B23" t="s">
         <v>26</v>
@@ -5352,7 +5356,7 @@
     </row>
     <row r="24" spans="1:19">
       <c r="A24" s="1" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="B24" t="s">
         <v>26</v>
@@ -5405,7 +5409,7 @@
     </row>
     <row r="25" spans="1:19">
       <c r="A25" s="1" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="B25" t="s">
         <v>26</v>
@@ -5458,7 +5462,7 @@
     </row>
     <row r="26" spans="1:19">
       <c r="A26" s="1" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="B26" t="s">
         <v>26</v>
@@ -5511,7 +5515,7 @@
     </row>
     <row r="27" spans="1:19">
       <c r="A27" s="1" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="B27" t="s">
         <v>26</v>
@@ -5564,7 +5568,7 @@
     </row>
     <row r="28" spans="1:19">
       <c r="A28" s="1" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="B28" t="s">
         <v>26</v>
@@ -5617,7 +5621,7 @@
     </row>
     <row r="29" spans="1:19">
       <c r="A29" s="1" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="B29" t="s">
         <v>26</v>
@@ -5670,7 +5674,7 @@
     </row>
     <row r="30" spans="1:19">
       <c r="A30" s="1" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="B30" t="s">
         <v>26</v>
@@ -5723,7 +5727,7 @@
     </row>
     <row r="31" spans="1:19">
       <c r="A31" s="1" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="B31" t="s">
         <v>26</v>
@@ -5776,7 +5780,7 @@
     </row>
     <row r="32" spans="1:19">
       <c r="A32" s="1" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="B32" t="s">
         <v>26</v>
@@ -5829,7 +5833,7 @@
     </row>
     <row r="33" spans="1:19">
       <c r="A33" s="1" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="B33" t="s">
         <v>26</v>
@@ -5882,7 +5886,7 @@
     </row>
     <row r="34" spans="1:19">
       <c r="A34" s="1" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="B34" t="s">
         <v>26</v>
@@ -5935,7 +5939,7 @@
     </row>
     <row r="35" spans="1:19">
       <c r="A35" s="1" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="B35" t="s">
         <v>26</v>
@@ -5988,7 +5992,7 @@
     </row>
     <row r="36" spans="1:19">
       <c r="A36" s="1" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="B36" t="s">
         <v>26</v>
@@ -6041,7 +6045,7 @@
     </row>
     <row r="37" spans="1:19">
       <c r="A37" s="1" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="B37" t="s">
         <v>26</v>
@@ -6094,7 +6098,7 @@
     </row>
     <row r="38" spans="1:19">
       <c r="A38" s="1" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="B38" t="s">
         <v>26</v>
@@ -6147,7 +6151,7 @@
     </row>
     <row r="39" spans="1:19">
       <c r="A39" s="1" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="B39" t="s">
         <v>26</v>
@@ -6200,7 +6204,7 @@
     </row>
     <row r="40" spans="1:19">
       <c r="A40" s="1" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="B40" t="s">
         <v>26</v>
@@ -6253,7 +6257,7 @@
     </row>
     <row r="41" spans="1:19">
       <c r="A41" s="1" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="B41" t="s">
         <v>26</v>
@@ -6306,7 +6310,7 @@
     </row>
     <row r="42" spans="1:19">
       <c r="A42" s="1" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="B42" t="s">
         <v>26</v>
@@ -6359,7 +6363,7 @@
     </row>
     <row r="43" spans="1:19">
       <c r="A43" s="1" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="B43" t="s">
         <v>26</v>
@@ -6412,7 +6416,7 @@
     </row>
     <row r="44" spans="1:19">
       <c r="A44" s="1" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="B44" t="s">
         <v>26</v>
@@ -6465,7 +6469,7 @@
     </row>
     <row r="45" spans="1:19">
       <c r="A45" s="1" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="B45" t="s">
         <v>26</v>
@@ -6518,7 +6522,7 @@
     </row>
     <row r="46" spans="1:19">
       <c r="A46" s="1" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="B46" t="s">
         <v>26</v>
@@ -6571,7 +6575,7 @@
     </row>
     <row r="47" spans="1:19">
       <c r="A47" s="1" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="B47" t="s">
         <v>26</v>
@@ -6624,7 +6628,7 @@
     </row>
     <row r="48" spans="1:19">
       <c r="A48" s="1" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="B48" t="s">
         <v>26</v>
@@ -6677,7 +6681,7 @@
     </row>
     <row r="49" spans="1:19">
       <c r="A49" s="1" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="B49" t="s">
         <v>26</v>
@@ -6730,7 +6734,7 @@
     </row>
     <row r="50" spans="1:19">
       <c r="A50" s="1" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="B50" t="s">
         <v>26</v>
@@ -6783,7 +6787,7 @@
     </row>
     <row r="51" spans="1:19">
       <c r="A51" s="1" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="B51" t="s">
         <v>26</v>
@@ -6836,7 +6840,7 @@
     </row>
     <row r="52" spans="1:19">
       <c r="A52" s="1" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="B52" t="s">
         <v>26</v>
@@ -6889,7 +6893,7 @@
     </row>
     <row r="53" spans="1:19">
       <c r="A53" s="1" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="B53" t="s">
         <v>26</v>
@@ -6942,7 +6946,7 @@
     </row>
     <row r="54" spans="1:19">
       <c r="A54" s="1" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="B54" t="s">
         <v>26</v>
@@ -6995,7 +6999,7 @@
     </row>
     <row r="55" spans="1:19">
       <c r="A55" s="1" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="B55" t="s">
         <v>26</v>
@@ -7048,7 +7052,7 @@
     </row>
     <row r="56" spans="1:19">
       <c r="A56" s="1" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="B56" t="s">
         <v>26</v>
@@ -7101,7 +7105,7 @@
     </row>
     <row r="57" spans="1:19">
       <c r="A57" s="1" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="B57" t="s">
         <v>26</v>
@@ -7154,7 +7158,7 @@
     </row>
     <row r="58" spans="1:19">
       <c r="A58" s="1" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="B58" t="s">
         <v>26</v>
@@ -7207,7 +7211,7 @@
     </row>
     <row r="59" spans="1:19">
       <c r="A59" s="1" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="B59" t="s">
         <v>26</v>
@@ -7260,7 +7264,7 @@
     </row>
     <row r="60" spans="1:19">
       <c r="A60" s="1" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
       <c r="B60" t="s">
         <v>26</v>
@@ -7313,7 +7317,7 @@
     </row>
     <row r="61" spans="1:19">
       <c r="A61" s="1" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="B61" t="s">
         <v>26</v>
@@ -7366,7 +7370,7 @@
     </row>
     <row r="62" spans="1:19">
       <c r="A62" s="1" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="B62" t="s">
         <v>26</v>
@@ -7419,7 +7423,7 @@
     </row>
     <row r="63" spans="1:19">
       <c r="A63" s="1" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="B63" t="s">
         <v>26</v>
@@ -7472,7 +7476,7 @@
     </row>
     <row r="64" spans="1:19">
       <c r="A64" s="1" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="B64" t="s">
         <v>26</v>
@@ -7525,7 +7529,7 @@
     </row>
     <row r="65" spans="1:19">
       <c r="A65" s="1" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
       <c r="B65" t="s">
         <v>26</v>
@@ -7578,7 +7582,7 @@
     </row>
     <row r="66" spans="1:19">
       <c r="A66" s="1" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
       <c r="B66" t="s">
         <v>26</v>
@@ -7631,7 +7635,7 @@
     </row>
     <row r="67" spans="1:19">
       <c r="A67" s="1" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="B67" t="s">
         <v>26</v>
@@ -7684,7 +7688,7 @@
     </row>
     <row r="68" spans="1:19">
       <c r="A68" s="1" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="B68" t="s">
         <v>26</v>
@@ -7737,7 +7741,7 @@
     </row>
     <row r="69" spans="1:19">
       <c r="A69" s="1" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="B69" t="s">
         <v>26</v>
@@ -7790,7 +7794,7 @@
     </row>
     <row r="70" spans="1:19">
       <c r="A70" s="1" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="B70" t="s">
         <v>26</v>
@@ -7843,7 +7847,7 @@
     </row>
     <row r="71" spans="1:19">
       <c r="A71" s="1" t="s">
-        <v>1219</v>
+        <v>1218</v>
       </c>
       <c r="B71" t="s">
         <v>26</v>
@@ -7896,7 +7900,7 @@
     </row>
     <row r="72" spans="1:19">
       <c r="A72" s="1" t="s">
-        <v>1220</v>
+        <v>1219</v>
       </c>
       <c r="B72" t="s">
         <v>26</v>
@@ -7949,7 +7953,7 @@
     </row>
     <row r="73" spans="1:19">
       <c r="A73" s="1" t="s">
-        <v>1221</v>
+        <v>1220</v>
       </c>
       <c r="B73" t="s">
         <v>26</v>
@@ -8002,7 +8006,7 @@
     </row>
     <row r="74" spans="1:19">
       <c r="A74" s="1" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
       <c r="B74" t="s">
         <v>26</v>
@@ -8055,7 +8059,7 @@
     </row>
     <row r="75" spans="1:19">
       <c r="A75" s="1" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
       <c r="B75" t="s">
         <v>26</v>
@@ -8108,7 +8112,7 @@
     </row>
     <row r="76" spans="1:19">
       <c r="A76" s="1" t="s">
-        <v>1224</v>
+        <v>1223</v>
       </c>
       <c r="B76" t="s">
         <v>26</v>
@@ -8161,7 +8165,7 @@
     </row>
     <row r="77" spans="1:19">
       <c r="A77" s="1" t="s">
-        <v>1225</v>
+        <v>1224</v>
       </c>
       <c r="B77" t="s">
         <v>26</v>
@@ -8214,7 +8218,7 @@
     </row>
     <row r="78" spans="1:19">
       <c r="A78" s="1" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
       <c r="B78" t="s">
         <v>26</v>
@@ -8267,7 +8271,7 @@
     </row>
     <row r="79" spans="1:19">
       <c r="A79" s="1" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="B79" t="s">
         <v>26</v>
@@ -8320,7 +8324,7 @@
     </row>
     <row r="80" spans="1:19">
       <c r="A80" s="1" t="s">
-        <v>1228</v>
+        <v>1227</v>
       </c>
       <c r="B80" t="s">
         <v>26</v>
@@ -8373,7 +8377,7 @@
     </row>
     <row r="81" spans="1:19">
       <c r="A81" s="1" t="s">
-        <v>1229</v>
+        <v>1228</v>
       </c>
       <c r="B81" t="s">
         <v>26</v>
@@ -8426,7 +8430,7 @@
     </row>
     <row r="82" spans="1:19">
       <c r="A82" s="1" t="s">
-        <v>1230</v>
+        <v>1229</v>
       </c>
       <c r="B82" t="s">
         <v>26</v>
@@ -8479,7 +8483,7 @@
     </row>
     <row r="83" spans="1:19">
       <c r="A83" s="1" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="B83" t="s">
         <v>26</v>
@@ -8532,7 +8536,7 @@
     </row>
     <row r="84" spans="1:19">
       <c r="A84" s="1" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
       <c r="B84" t="s">
         <v>26</v>
@@ -8585,7 +8589,7 @@
     </row>
     <row r="85" spans="1:19">
       <c r="A85" s="1" t="s">
-        <v>1233</v>
+        <v>1232</v>
       </c>
       <c r="B85" t="s">
         <v>26</v>
@@ -8638,7 +8642,7 @@
     </row>
     <row r="86" spans="1:19">
       <c r="A86" s="1" t="s">
-        <v>1234</v>
+        <v>1233</v>
       </c>
       <c r="B86" t="s">
         <v>26</v>
@@ -8694,7 +8698,7 @@
     </row>
     <row r="87" spans="1:19">
       <c r="A87" s="1" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
       <c r="B87" t="s">
         <v>26</v>
@@ -8747,7 +8751,7 @@
     </row>
     <row r="88" spans="1:19">
       <c r="A88" s="1" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="B88" t="s">
         <v>26</v>
@@ -8800,7 +8804,7 @@
     </row>
     <row r="89" spans="1:19">
       <c r="A89" s="1" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="B89" t="s">
         <v>26</v>
@@ -8853,7 +8857,7 @@
     </row>
     <row r="90" spans="1:19">
       <c r="A90" s="1" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
       <c r="B90" t="s">
         <v>26</v>
@@ -8906,7 +8910,7 @@
     </row>
     <row r="91" spans="1:19">
       <c r="A91" s="1" t="s">
-        <v>1239</v>
+        <v>1238</v>
       </c>
       <c r="B91" t="s">
         <v>26</v>
@@ -8959,7 +8963,7 @@
     </row>
     <row r="92" spans="1:19">
       <c r="A92" s="1" t="s">
-        <v>1240</v>
+        <v>1239</v>
       </c>
       <c r="B92" t="s">
         <v>26</v>
@@ -9012,7 +9016,7 @@
     </row>
     <row r="93" spans="1:19">
       <c r="A93" s="1" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="B93" t="s">
         <v>26</v>
@@ -9065,7 +9069,7 @@
     </row>
     <row r="94" spans="1:19">
       <c r="A94" s="1" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
       <c r="B94" t="s">
         <v>26</v>
@@ -9118,7 +9122,7 @@
     </row>
     <row r="95" spans="1:19">
       <c r="A95" s="1" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
       <c r="B95" t="s">
         <v>26</v>
@@ -9171,7 +9175,7 @@
     </row>
     <row r="96" spans="1:19">
       <c r="A96" s="1" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="B96" t="s">
         <v>26</v>
@@ -9224,7 +9228,7 @@
     </row>
     <row r="97" spans="1:19">
       <c r="A97" s="1" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="B97" t="s">
         <v>26</v>
@@ -9280,7 +9284,7 @@
     </row>
     <row r="98" spans="1:19">
       <c r="A98" s="1" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="B98" t="s">
         <v>26</v>
@@ -9333,7 +9337,7 @@
     </row>
     <row r="99" spans="1:19">
       <c r="A99" s="1" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="B99" t="s">
         <v>26</v>
@@ -9386,7 +9390,7 @@
     </row>
     <row r="100" spans="1:19">
       <c r="A100" s="1" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
       <c r="B100" t="s">
         <v>26</v>
@@ -9439,7 +9443,7 @@
     </row>
     <row r="101" spans="1:19">
       <c r="A101" s="1" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="B101" t="s">
         <v>26</v>
@@ -9492,7 +9496,7 @@
     </row>
     <row r="102" spans="1:19">
       <c r="A102" s="1" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
       <c r="B102" t="s">
         <v>26</v>
@@ -9545,7 +9549,7 @@
     </row>
     <row r="103" spans="1:19">
       <c r="A103" s="1" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
       <c r="B103" t="s">
         <v>26</v>
@@ -9598,7 +9602,7 @@
     </row>
     <row r="104" spans="1:19">
       <c r="A104" s="1" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="B104" t="s">
         <v>26</v>
@@ -9651,7 +9655,7 @@
     </row>
     <row r="105" spans="1:19">
       <c r="A105" s="1" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="B105" t="s">
         <v>26</v>
@@ -9704,7 +9708,7 @@
     </row>
     <row r="106" spans="1:19">
       <c r="A106" s="1" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="B106" t="s">
         <v>26</v>
@@ -9757,7 +9761,7 @@
     </row>
     <row r="107" spans="1:19">
       <c r="A107" s="1" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
       <c r="B107" t="s">
         <v>26</v>
@@ -9810,7 +9814,7 @@
     </row>
     <row r="108" spans="1:19">
       <c r="A108" s="1" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
       <c r="B108" t="s">
         <v>26</v>

</xml_diff>